<commit_message>
feat(6365): populate SOTP Valuation Cross-Check with DCF/Comps values
- PGM: YEN 7,391 (+42.5% vs SOTP Base)
- Exit Multiple: YEN 8,846 (+70.6%)
- Comps EV/EBITDA: YEN 8,200 (+58.1%)
- Comps PER: YEN 7,496 (+44.5%)
- SOTP Base: YEN 5,186

Values computed by opening 6365_DCF_Model_20260411.xlsx via Excel COM,
reading computed share prices from DCF Model C55/C64 and Comps Analysis C27/C28.
</commit_message>
<xml_diff>
--- a/models/6365_SOTP_Model.xlsx
+++ b/models/6365_SOTP_Model.xlsx
@@ -718,7 +718,9 @@
           <t>DCF — Perpetuity Growth</t>
         </is>
       </c>
-      <c r="C13" s="9" t="n"/>
+      <c r="C13" s="9" t="n">
+        <v>7391</v>
+      </c>
       <c r="D13" s="10">
         <f>(C13-$C$12)/$C$12</f>
         <v/>
@@ -730,7 +732,9 @@
           <t>DCF — Exit Multiple</t>
         </is>
       </c>
-      <c r="C14" s="9" t="n"/>
+      <c r="C14" s="9" t="n">
+        <v>8846</v>
+      </c>
       <c r="D14" s="10">
         <f>(C14-$C$12)/$C$12</f>
         <v/>
@@ -742,7 +746,9 @@
           <t>Comps — EV/EBITDA</t>
         </is>
       </c>
-      <c r="C15" s="9" t="n"/>
+      <c r="C15" s="9" t="n">
+        <v>8200</v>
+      </c>
       <c r="D15" s="10">
         <f>(C15-$C$12)/$C$12</f>
         <v/>
@@ -754,7 +760,9 @@
           <t>Comps — PER</t>
         </is>
       </c>
-      <c r="C16" s="9" t="n"/>
+      <c r="C16" s="9" t="n">
+        <v>7496</v>
+      </c>
       <c r="D16" s="10">
         <f>(C16-$C$12)/$C$12</f>
         <v/>

</xml_diff>